<commit_message>
Add PART (item card) field catalog and align ITEMS mapping
- specs/PART.yaml — קטלוג 219 שדות ממסך כרטיס פריט (אכיפה אוטומטית של
  אורך/חובה/טיפוס/דיוק/בוליאני)
- mappings/ITEMS.yaml עודכן לשדות התקניים: PARTNAME/PARTDES/STATDES/TYPE
  (P/R/O)/UNITNAME/PUNITNAME/CONV/FAMILYNAME/BARCODE/PURPRICE
- קובץ הדוגמה items.xlsx עודכן לקודי משפחה קצרים (רוחב 8) ועמודת טיפוס

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012r2WeiXLPPMNzZnbMvw2z7
</commit_message>
<xml_diff>
--- a/file-loader/examples/items.xlsx
+++ b/file-loader/examples/items.xlsx
@@ -439,17 +439,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>טיפוס</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>ברקוד</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>מחיר</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>לא פעיל</t>
         </is>
       </c>
     </row>
@@ -466,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>מוצרי מדף</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -476,17 +476,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>קניה</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>7290001000017</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1.50</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>פעיל</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>מוצרי מדף</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -513,17 +513,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>קניה</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>7290001000024</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>0.9</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>פעיל</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>חשמל</t>
+          <t>20</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -550,17 +550,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>קניה</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>7290001000031</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>4.25</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>פעיל</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>צבעים</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -587,17 +587,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>ייצור</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>7290001000048</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>38.90</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>לא פעיל</t>
         </is>
       </c>
     </row>
@@ -614,7 +614,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>בניין</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -624,17 +624,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>קניה</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>7290001000055</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>0.75</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>פעיל</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>כללי</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -657,17 +657,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>קניה</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>7290001000062</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>10</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>פעיל</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>כללי</t>
+          <t>10</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -694,17 +694,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>קניה</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>7290001000079</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>בדיקה</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>פעיל</t>
         </is>
       </c>
     </row>

</xml_diff>